<commit_message>
JLF: Correction mise en place onglet température
</commit_message>
<xml_diff>
--- a/docs/ChronoStageTutoré_2026.1b.xlsx
+++ b/docs/ChronoStageTutoré_2026.1b.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lefur\Documents\GitHub\MIAGE-2026\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB75102E-0D1C-4D66-9D27-EC452B685006}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A61A29C2-8C13-44D4-8C9B-3B1C1CAAE648}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="24669" windowHeight="9797" xr2:uid="{8CD262DD-37D0-4D54-B340-C5BBE90D80FB}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="44">
   <si>
     <t>Date</t>
   </si>
@@ -91,13 +91,91 @@
   </si>
   <si>
     <t>contextCreator</t>
+  </si>
+  <si>
+    <t>Fix: add image + Style2dTemperature + try to draw temperature changes</t>
+  </si>
+  <si>
+    <t>corrections tuteur (voir mail)</t>
+  </si>
+  <si>
+    <t>scenario.xml</t>
+  </si>
+  <si>
+    <t>constructeur C_Protocol_PNMC_temperature</t>
+  </si>
+  <si>
+    <t>ajout de couleurs et distinction terre dans manageOneEvent :</t>
+  </si>
+  <si>
+    <t>));</t>
+  </si>
+  <si>
+    <t>255,19,0</t>
+  </si>
+  <si>
+    <t>, new Color(</t>
+  </si>
+  <si>
+    <t>colorMap.put(</t>
+  </si>
+  <si>
+    <r>
+      <t>255,</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>66,0</t>
+    </r>
+  </si>
+  <si>
+    <t>255,103,0</t>
+  </si>
+  <si>
+    <t>255,150,0</t>
+  </si>
+  <si>
+    <t>255,191,0</t>
+  </si>
+  <si>
+    <t>255,235,0</t>
+  </si>
+  <si>
+    <t>234,243,16</t>
+  </si>
+  <si>
+    <t>190,218,49</t>
+  </si>
+  <si>
+    <t>146,194,82</t>
+  </si>
+  <si>
+    <t>104,171,113</t>
+  </si>
+  <si>
+    <t>62,146,146</t>
+  </si>
+  <si>
+    <t>21,124,176</t>
+  </si>
+  <si>
+    <t>copié dans C_Style2dTemperature#colorMapTemperature</t>
+  </si>
+  <si>
+    <t>ajout de test PNMC_TEMPERATURE dans C_Protocol_PNMC_drifters</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -115,6 +193,27 @@
     <font>
       <b/>
       <sz val="18"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -147,11 +246,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -466,17 +572,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50A5B30A-9091-4023-BC8F-85B7675FB373}">
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:K29"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.3828125" defaultRowHeight="18.45" x14ac:dyDescent="0.5"/>
   <cols>
     <col min="1" max="1" width="17.69140625" style="1" customWidth="1"/>
     <col min="2" max="2" width="43.69140625" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="36.3046875" style="1" customWidth="1"/>
     <col min="4" max="4" width="102.15234375" style="1" customWidth="1"/>
-    <col min="5" max="16384" width="11.3828125" style="1"/>
+    <col min="5" max="5" width="12.69140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="2.84375" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.765625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.84375" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="2.61328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.3828125" style="1"/>
+    <col min="11" max="11" width="35.61328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="16384" width="11.3828125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="23.15" x14ac:dyDescent="0.6">
+    <row r="1" spans="1:11" ht="23.15" x14ac:dyDescent="0.6">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -490,7 +603,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.5">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A2" s="2">
         <v>46108</v>
       </c>
@@ -501,7 +614,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.5">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A3" s="2">
         <v>46119</v>
       </c>
@@ -512,7 +625,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.5">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A4" s="2">
         <v>46119</v>
       </c>
@@ -523,7 +636,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.5">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A5" s="2">
         <v>46121</v>
       </c>
@@ -534,7 +647,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.5">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A6" s="2">
         <v>46121</v>
       </c>
@@ -545,7 +658,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.5">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A7" s="2">
         <v>46129</v>
       </c>
@@ -556,7 +669,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.5">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A8" s="2">
         <v>46135</v>
       </c>
@@ -567,29 +680,329 @@
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.5">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.5">
       <c r="C9" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.5">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.5">
       <c r="C10" s="1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.5">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.5">
       <c r="C11" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.5">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.5">
       <c r="C12" s="1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.5">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.5">
       <c r="C13" s="1" t="s">
         <v>21</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.5">
+      <c r="A14" s="2">
+        <v>46023</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.5">
+      <c r="A15" s="2">
+        <v>46146</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.5">
+      <c r="C16" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="K16" s="6" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="17" spans="3:11" x14ac:dyDescent="0.5">
+      <c r="C17" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="K17" s="6"/>
+    </row>
+    <row r="18" spans="3:11" x14ac:dyDescent="0.5">
+      <c r="C18" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E18" t="s">
+        <v>30</v>
+      </c>
+      <c r="F18">
+        <v>1</v>
+      </c>
+      <c r="G18" t="s">
+        <v>29</v>
+      </c>
+      <c r="H18" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="I18" t="s">
+        <v>27</v>
+      </c>
+      <c r="J18"/>
+      <c r="K18" t="str">
+        <f>+E18&amp;F18&amp;G18&amp;H18&amp;I18</f>
+        <v>colorMap.put(1, new Color(21,124,176));</v>
+      </c>
+    </row>
+    <row r="19" spans="3:11" x14ac:dyDescent="0.5">
+      <c r="E19" t="s">
+        <v>30</v>
+      </c>
+      <c r="F19">
+        <v>2</v>
+      </c>
+      <c r="G19" t="s">
+        <v>29</v>
+      </c>
+      <c r="H19" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="I19" t="s">
+        <v>27</v>
+      </c>
+      <c r="J19"/>
+      <c r="K19" t="str">
+        <f>+E19&amp;F19&amp;G19&amp;H19&amp;I19</f>
+        <v>colorMap.put(2, new Color(62,146,146));</v>
+      </c>
+    </row>
+    <row r="20" spans="3:11" x14ac:dyDescent="0.5">
+      <c r="E20" t="s">
+        <v>30</v>
+      </c>
+      <c r="F20">
+        <v>3</v>
+      </c>
+      <c r="G20" t="s">
+        <v>29</v>
+      </c>
+      <c r="H20" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="I20" t="s">
+        <v>27</v>
+      </c>
+      <c r="J20"/>
+      <c r="K20" t="str">
+        <f>+E20&amp;F20&amp;G20&amp;H20&amp;I20</f>
+        <v>colorMap.put(3, new Color(104,171,113));</v>
+      </c>
+    </row>
+    <row r="21" spans="3:11" x14ac:dyDescent="0.5">
+      <c r="E21" t="s">
+        <v>30</v>
+      </c>
+      <c r="F21">
+        <v>4</v>
+      </c>
+      <c r="G21" t="s">
+        <v>29</v>
+      </c>
+      <c r="H21" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="I21" t="s">
+        <v>27</v>
+      </c>
+      <c r="J21"/>
+      <c r="K21" t="str">
+        <f>+E21&amp;F21&amp;G21&amp;H21&amp;I21</f>
+        <v>colorMap.put(4, new Color(146,194,82));</v>
+      </c>
+    </row>
+    <row r="22" spans="3:11" x14ac:dyDescent="0.5">
+      <c r="E22" t="s">
+        <v>30</v>
+      </c>
+      <c r="F22">
+        <v>5</v>
+      </c>
+      <c r="G22" t="s">
+        <v>29</v>
+      </c>
+      <c r="H22" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="I22" t="s">
+        <v>27</v>
+      </c>
+      <c r="J22"/>
+      <c r="K22" t="str">
+        <f>+E22&amp;F22&amp;G22&amp;H22&amp;I22</f>
+        <v>colorMap.put(5, new Color(190,218,49));</v>
+      </c>
+    </row>
+    <row r="23" spans="3:11" x14ac:dyDescent="0.5">
+      <c r="E23" t="s">
+        <v>30</v>
+      </c>
+      <c r="F23">
+        <v>6</v>
+      </c>
+      <c r="G23" t="s">
+        <v>29</v>
+      </c>
+      <c r="H23" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="I23" t="s">
+        <v>27</v>
+      </c>
+      <c r="J23"/>
+      <c r="K23" t="str">
+        <f>+E23&amp;F23&amp;G23&amp;H23&amp;I23</f>
+        <v>colorMap.put(6, new Color(234,243,16));</v>
+      </c>
+    </row>
+    <row r="24" spans="3:11" x14ac:dyDescent="0.5">
+      <c r="E24" t="s">
+        <v>30</v>
+      </c>
+      <c r="F24">
+        <v>7</v>
+      </c>
+      <c r="G24" t="s">
+        <v>29</v>
+      </c>
+      <c r="H24" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="I24" t="s">
+        <v>27</v>
+      </c>
+      <c r="J24"/>
+      <c r="K24" t="str">
+        <f>+E24&amp;F24&amp;G24&amp;H24&amp;I24</f>
+        <v>colorMap.put(7, new Color(255,235,0));</v>
+      </c>
+    </row>
+    <row r="25" spans="3:11" x14ac:dyDescent="0.5">
+      <c r="E25" t="s">
+        <v>30</v>
+      </c>
+      <c r="F25">
+        <v>8</v>
+      </c>
+      <c r="G25" t="s">
+        <v>29</v>
+      </c>
+      <c r="H25" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="I25" t="s">
+        <v>27</v>
+      </c>
+      <c r="J25"/>
+      <c r="K25" t="str">
+        <f>+E25&amp;F25&amp;G25&amp;H25&amp;I25</f>
+        <v>colorMap.put(8, new Color(255,191,0));</v>
+      </c>
+    </row>
+    <row r="26" spans="3:11" x14ac:dyDescent="0.5">
+      <c r="E26" t="s">
+        <v>30</v>
+      </c>
+      <c r="F26">
+        <v>9</v>
+      </c>
+      <c r="G26" t="s">
+        <v>29</v>
+      </c>
+      <c r="H26" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="I26" t="s">
+        <v>27</v>
+      </c>
+      <c r="J26"/>
+      <c r="K26" t="str">
+        <f>+E26&amp;F26&amp;G26&amp;H26&amp;I26</f>
+        <v>colorMap.put(9, new Color(255,150,0));</v>
+      </c>
+    </row>
+    <row r="27" spans="3:11" x14ac:dyDescent="0.5">
+      <c r="E27" t="s">
+        <v>30</v>
+      </c>
+      <c r="F27">
+        <v>10</v>
+      </c>
+      <c r="G27" t="s">
+        <v>29</v>
+      </c>
+      <c r="H27" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="I27" t="s">
+        <v>27</v>
+      </c>
+      <c r="J27"/>
+      <c r="K27" t="str">
+        <f>+E27&amp;F27&amp;G27&amp;H27&amp;I27</f>
+        <v>colorMap.put(10, new Color(255,103,0));</v>
+      </c>
+    </row>
+    <row r="28" spans="3:11" x14ac:dyDescent="0.5">
+      <c r="E28" t="s">
+        <v>30</v>
+      </c>
+      <c r="F28">
+        <v>11</v>
+      </c>
+      <c r="G28" t="s">
+        <v>29</v>
+      </c>
+      <c r="H28" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="I28" t="s">
+        <v>27</v>
+      </c>
+      <c r="J28"/>
+      <c r="K28" t="str">
+        <f>+E28&amp;F28&amp;G28&amp;H28&amp;I28</f>
+        <v>colorMap.put(11, new Color(255,66,0));</v>
+      </c>
+    </row>
+    <row r="29" spans="3:11" x14ac:dyDescent="0.5">
+      <c r="E29" t="s">
+        <v>30</v>
+      </c>
+      <c r="F29">
+        <v>12</v>
+      </c>
+      <c r="G29" t="s">
+        <v>29</v>
+      </c>
+      <c r="H29" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="I29" t="s">
+        <v>27</v>
+      </c>
+      <c r="J29"/>
+      <c r="K29" t="str">
+        <f>+E29&amp;F29&amp;G29&amp;H29&amp;I29</f>
+        <v>colorMap.put(12, new Color(255,19,0));</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ajout javadoc et update chronoStage
</commit_message>
<xml_diff>
--- a/docs/ChronoStageTutoré_2026.1b.xlsx
+++ b/docs/ChronoStageTutoré_2026.1b.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lefur\Documents\GitHub\MIAGE-2026\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A61A29C2-8C13-44D4-8C9B-3B1C1CAAE648}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E934FDBE-E228-4FF1-BAF8-3CA65F11FAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="24669" windowHeight="9797" xr2:uid="{8CD262DD-37D0-4D54-B340-C5BBE90D80FB}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{8CD262DD-37D0-4D54-B340-C5BBE90D80FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="48">
   <si>
     <t>Date</t>
   </si>
@@ -169,6 +169,18 @@
   </si>
   <si>
     <t>ajout de test PNMC_TEMPERATURE dans C_Protocol_PNMC_drifters</t>
+  </si>
+  <si>
+    <t>Checking protocol temperature</t>
+  </si>
+  <si>
+    <t>Lecture et validation des corrections tuteur</t>
+  </si>
+  <si>
+    <t>écriture javadoc C_Protocol_PNMC_temperature (constructeur et manageOneEvent)</t>
+  </si>
+  <si>
+    <t>réponse mail des étudiants au tuteur pour confirmer la possible modification du GUI (onglets de droite)</t>
   </si>
 </sst>
 </file>
@@ -572,24 +584,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50A5B30A-9091-4023-BC8F-85B7675FB373}">
-  <dimension ref="A1:K29"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.3828125" defaultRowHeight="18.45" x14ac:dyDescent="0.5"/>
+  <dimension ref="A1:K32"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.69140625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="43.69140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="36.3046875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="102.15234375" style="1" customWidth="1"/>
-    <col min="5" max="5" width="12.69140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="2.84375" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.765625" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.84375" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="2.61328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.3828125" style="1"/>
-    <col min="11" max="11" width="35.61328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="16384" width="11.3828125" style="1"/>
+    <col min="1" max="1" width="17.7109375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="43.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="96.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="102.140625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="12.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="2.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="2.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.42578125" style="1"/>
+    <col min="11" max="11" width="35.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="16384" width="11.42578125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="23.15" x14ac:dyDescent="0.6">
+    <row r="1" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -603,7 +615,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
         <v>46108</v>
       </c>
@@ -614,7 +626,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
         <v>46119</v>
       </c>
@@ -625,7 +637,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
         <v>46119</v>
       </c>
@@ -636,7 +648,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
         <v>46121</v>
       </c>
@@ -647,7 +659,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <v>46121</v>
       </c>
@@ -658,7 +670,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
         <v>46129</v>
       </c>
@@ -669,7 +681,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
         <v>46135</v>
       </c>
@@ -680,32 +692,32 @@
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="C9" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="C10" s="1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="C11" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="C12" s="1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="C13" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" s="2">
         <v>46023</v>
       </c>
@@ -713,7 +725,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" s="2">
         <v>46146</v>
       </c>
@@ -724,7 +736,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.5">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="C16" s="1" t="s">
         <v>25</v>
       </c>
@@ -732,13 +744,13 @@
         <v>42</v>
       </c>
     </row>
-    <row r="17" spans="3:11" x14ac:dyDescent="0.5">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="C17" s="1" t="s">
         <v>43</v>
       </c>
       <c r="K17" s="6"/>
     </row>
-    <row r="18" spans="3:11" x14ac:dyDescent="0.5">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="C18" s="1" t="s">
         <v>26</v>
       </c>
@@ -759,11 +771,11 @@
       </c>
       <c r="J18"/>
       <c r="K18" t="str">
-        <f>+E18&amp;F18&amp;G18&amp;H18&amp;I18</f>
+        <f t="shared" ref="K18:K29" si="0">+E18&amp;F18&amp;G18&amp;H18&amp;I18</f>
         <v>colorMap.put(1, new Color(21,124,176));</v>
       </c>
     </row>
-    <row r="19" spans="3:11" x14ac:dyDescent="0.5">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="E19" t="s">
         <v>30</v>
       </c>
@@ -781,11 +793,11 @@
       </c>
       <c r="J19"/>
       <c r="K19" t="str">
-        <f>+E19&amp;F19&amp;G19&amp;H19&amp;I19</f>
+        <f t="shared" si="0"/>
         <v>colorMap.put(2, new Color(62,146,146));</v>
       </c>
     </row>
-    <row r="20" spans="3:11" x14ac:dyDescent="0.5">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="E20" t="s">
         <v>30</v>
       </c>
@@ -803,11 +815,11 @@
       </c>
       <c r="J20"/>
       <c r="K20" t="str">
-        <f>+E20&amp;F20&amp;G20&amp;H20&amp;I20</f>
+        <f t="shared" si="0"/>
         <v>colorMap.put(3, new Color(104,171,113));</v>
       </c>
     </row>
-    <row r="21" spans="3:11" x14ac:dyDescent="0.5">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="E21" t="s">
         <v>30</v>
       </c>
@@ -825,11 +837,11 @@
       </c>
       <c r="J21"/>
       <c r="K21" t="str">
-        <f>+E21&amp;F21&amp;G21&amp;H21&amp;I21</f>
+        <f t="shared" si="0"/>
         <v>colorMap.put(4, new Color(146,194,82));</v>
       </c>
     </row>
-    <row r="22" spans="3:11" x14ac:dyDescent="0.5">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="E22" t="s">
         <v>30</v>
       </c>
@@ -847,11 +859,11 @@
       </c>
       <c r="J22"/>
       <c r="K22" t="str">
-        <f>+E22&amp;F22&amp;G22&amp;H22&amp;I22</f>
+        <f t="shared" si="0"/>
         <v>colorMap.put(5, new Color(190,218,49));</v>
       </c>
     </row>
-    <row r="23" spans="3:11" x14ac:dyDescent="0.5">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="E23" t="s">
         <v>30</v>
       </c>
@@ -869,11 +881,11 @@
       </c>
       <c r="J23"/>
       <c r="K23" t="str">
-        <f>+E23&amp;F23&amp;G23&amp;H23&amp;I23</f>
+        <f t="shared" si="0"/>
         <v>colorMap.put(6, new Color(234,243,16));</v>
       </c>
     </row>
-    <row r="24" spans="3:11" x14ac:dyDescent="0.5">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="E24" t="s">
         <v>30</v>
       </c>
@@ -891,11 +903,11 @@
       </c>
       <c r="J24"/>
       <c r="K24" t="str">
-        <f>+E24&amp;F24&amp;G24&amp;H24&amp;I24</f>
+        <f t="shared" si="0"/>
         <v>colorMap.put(7, new Color(255,235,0));</v>
       </c>
     </row>
-    <row r="25" spans="3:11" x14ac:dyDescent="0.5">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="E25" t="s">
         <v>30</v>
       </c>
@@ -913,11 +925,11 @@
       </c>
       <c r="J25"/>
       <c r="K25" t="str">
-        <f>+E25&amp;F25&amp;G25&amp;H25&amp;I25</f>
+        <f t="shared" si="0"/>
         <v>colorMap.put(8, new Color(255,191,0));</v>
       </c>
     </row>
-    <row r="26" spans="3:11" x14ac:dyDescent="0.5">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="E26" t="s">
         <v>30</v>
       </c>
@@ -935,11 +947,11 @@
       </c>
       <c r="J26"/>
       <c r="K26" t="str">
-        <f>+E26&amp;F26&amp;G26&amp;H26&amp;I26</f>
+        <f t="shared" si="0"/>
         <v>colorMap.put(9, new Color(255,150,0));</v>
       </c>
     </row>
-    <row r="27" spans="3:11" x14ac:dyDescent="0.5">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="E27" t="s">
         <v>30</v>
       </c>
@@ -957,11 +969,11 @@
       </c>
       <c r="J27"/>
       <c r="K27" t="str">
-        <f>+E27&amp;F27&amp;G27&amp;H27&amp;I27</f>
+        <f t="shared" si="0"/>
         <v>colorMap.put(10, new Color(255,103,0));</v>
       </c>
     </row>
-    <row r="28" spans="3:11" x14ac:dyDescent="0.5">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="E28" t="s">
         <v>30</v>
       </c>
@@ -979,11 +991,11 @@
       </c>
       <c r="J28"/>
       <c r="K28" t="str">
-        <f>+E28&amp;F28&amp;G28&amp;H28&amp;I28</f>
+        <f t="shared" si="0"/>
         <v>colorMap.put(11, new Color(255,66,0));</v>
       </c>
     </row>
-    <row r="29" spans="3:11" x14ac:dyDescent="0.5">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="E29" t="s">
         <v>30</v>
       </c>
@@ -1001,8 +1013,29 @@
       </c>
       <c r="J29"/>
       <c r="K29" t="str">
-        <f>+E29&amp;F29&amp;G29&amp;H29&amp;I29</f>
+        <f t="shared" si="0"/>
         <v>colorMap.put(12, new Color(255,19,0));</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A30" s="2">
+        <v>46149</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="C31" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="C32" s="1" t="s">
+        <v>47</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Décorations complémentaires pour le protocole température
</commit_message>
<xml_diff>
--- a/docs/ChronoStageTutoré_2026.1b.xlsx
+++ b/docs/ChronoStageTutoré_2026.1b.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lefur\Documents\GitHub\MIAGE-2026\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E934FDBE-E228-4FF1-BAF8-3CA65F11FAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F7ABED8-87CD-41E8-8B6D-D62D36EF589F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{8CD262DD-37D0-4D54-B340-C5BBE90D80FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="49">
   <si>
     <t>Date</t>
   </si>
@@ -181,6 +181,9 @@
   </si>
   <si>
     <t>réponse mail des étudiants au tuteur pour confirmer la possible modification du GUI (onglets de droite)</t>
+  </si>
+  <si>
+    <t>ajout/modification de décorations</t>
   </si>
 </sst>
 </file>
@@ -584,24 +587,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50A5B30A-9091-4023-BC8F-85B7675FB373}">
-  <dimension ref="A1:K32"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:K33"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.3828125" defaultRowHeight="18.45" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="1" width="17.7109375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="43.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="96.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="102.140625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="12.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="2.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="2.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.42578125" style="1"/>
-    <col min="11" max="11" width="35.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="16384" width="11.42578125" style="1"/>
+    <col min="1" max="1" width="17.69140625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="43.69140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="96.3046875" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="102.15234375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="12.69140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="2.84375" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.69140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.84375" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="2.53515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.3828125" style="1"/>
+    <col min="11" max="11" width="35.53515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="16384" width="11.3828125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" ht="23.15" x14ac:dyDescent="0.6">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -615,7 +618,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A2" s="2">
         <v>46108</v>
       </c>
@@ -626,7 +629,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A3" s="2">
         <v>46119</v>
       </c>
@@ -637,7 +640,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A4" s="2">
         <v>46119</v>
       </c>
@@ -648,7 +651,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A5" s="2">
         <v>46121</v>
       </c>
@@ -659,7 +662,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A6" s="2">
         <v>46121</v>
       </c>
@@ -670,7 +673,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A7" s="2">
         <v>46129</v>
       </c>
@@ -681,7 +684,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A8" s="2">
         <v>46135</v>
       </c>
@@ -692,32 +695,32 @@
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.5">
       <c r="C9" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.5">
       <c r="C10" s="1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.5">
       <c r="C11" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.5">
       <c r="C12" s="1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.5">
       <c r="C13" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A14" s="2">
         <v>46023</v>
       </c>
@@ -725,7 +728,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A15" s="2">
         <v>46146</v>
       </c>
@@ -736,7 +739,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.5">
       <c r="C16" s="1" t="s">
         <v>25</v>
       </c>
@@ -744,13 +747,13 @@
         <v>42</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.5">
       <c r="C17" s="1" t="s">
         <v>43</v>
       </c>
       <c r="K17" s="6"/>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.5">
       <c r="C18" s="1" t="s">
         <v>26</v>
       </c>
@@ -775,7 +778,7 @@
         <v>colorMap.put(1, new Color(21,124,176));</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.5">
       <c r="E19" t="s">
         <v>30</v>
       </c>
@@ -797,7 +800,7 @@
         <v>colorMap.put(2, new Color(62,146,146));</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.5">
       <c r="E20" t="s">
         <v>30</v>
       </c>
@@ -819,7 +822,7 @@
         <v>colorMap.put(3, new Color(104,171,113));</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.5">
       <c r="E21" t="s">
         <v>30</v>
       </c>
@@ -841,7 +844,7 @@
         <v>colorMap.put(4, new Color(146,194,82));</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.5">
       <c r="E22" t="s">
         <v>30</v>
       </c>
@@ -863,7 +866,7 @@
         <v>colorMap.put(5, new Color(190,218,49));</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.5">
       <c r="E23" t="s">
         <v>30</v>
       </c>
@@ -885,7 +888,7 @@
         <v>colorMap.put(6, new Color(234,243,16));</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.5">
       <c r="E24" t="s">
         <v>30</v>
       </c>
@@ -907,7 +910,7 @@
         <v>colorMap.put(7, new Color(255,235,0));</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.5">
       <c r="E25" t="s">
         <v>30</v>
       </c>
@@ -929,7 +932,7 @@
         <v>colorMap.put(8, new Color(255,191,0));</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.5">
       <c r="E26" t="s">
         <v>30</v>
       </c>
@@ -951,7 +954,7 @@
         <v>colorMap.put(9, new Color(255,150,0));</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.5">
       <c r="E27" t="s">
         <v>30</v>
       </c>
@@ -973,7 +976,7 @@
         <v>colorMap.put(10, new Color(255,103,0));</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.5">
       <c r="E28" t="s">
         <v>30</v>
       </c>
@@ -995,7 +998,7 @@
         <v>colorMap.put(11, new Color(255,66,0));</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.5">
       <c r="E29" t="s">
         <v>30</v>
       </c>
@@ -1017,7 +1020,7 @@
         <v>colorMap.put(12, new Color(255,19,0));</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.5">
       <c r="A30" s="2">
         <v>46149</v>
       </c>
@@ -1028,14 +1031,22 @@
         <v>45</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.5">
       <c r="C31" s="1" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.5">
       <c r="C32" s="1" t="s">
         <v>47</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.5">
+      <c r="A33" s="2">
+        <v>46153</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>